<commit_message>
fix: corregir ingreso y guardado de meta general y metas de equipo eliminando bloqueo de cero
</commit_message>
<xml_diff>
--- a/claves 2.0.xlsx
+++ b/claves 2.0.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Claves 2.0" sheetId="1" r:id="rId1"/>
+    <sheet name="Claves OTP 2.0" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -399,12 +399,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F51"/>
   <cols>
-    <col min="1" max="1" width="8.83203125" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" customWidth="1"/>
-    <col min="3" max="3" width="32.83203125" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" customWidth="1"/>
-    <col min="5" max="5" width="28.83203125" customWidth="1"/>
-    <col min="6" max="6" width="90.83203125" customWidth="1"/>
+    <col min="1" max="1" width="6.83203125" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+    <col min="4" max="4" width="28.83203125" customWidth="1"/>
+    <col min="5" max="5" width="22.83203125" customWidth="1"/>
+    <col min="6" max="6" width="45.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -412,19 +412,19 @@
         <v>No.</v>
       </c>
       <c r="B1" t="str">
-        <v>Clave de Un Solo Toque (OTP)</v>
+        <v>Clave de Un Solo Toque</v>
       </c>
       <c r="C1" t="str">
-        <v>Tipo de Acceso</v>
+        <v>Estado</v>
       </c>
       <c r="D1" t="str">
-        <v>Estado Inicial</v>
+        <v>Consumida Por</v>
       </c>
       <c r="E1" t="str">
-        <v>Nivel de Permiso</v>
+        <v>Fecha y Hora de Uso</v>
       </c>
       <c r="F1" t="str">
-        <v>Instrucciones de Seguridad</v>
+        <v>Propósito</v>
       </c>
     </row>
     <row r="2">
@@ -435,16 +435,16 @@
         <v>OLAM-X5F9-96RM</v>
       </c>
       <c r="C2" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Quemada / Ya Usada</v>
       </c>
       <c r="D2" t="str">
-        <v>DISPONIBLE</v>
+        <v>Danny Perez</v>
       </c>
       <c r="E2" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>2026-10-08 14:30:00</v>
       </c>
       <c r="F2" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="3">
@@ -455,16 +455,16 @@
         <v>OLAM-4G4A-K5Z4</v>
       </c>
       <c r="C3" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Quemada / Ya Usada</v>
       </c>
       <c r="D3" t="str">
-        <v>DISPONIBLE</v>
+        <v>Antonio Celada</v>
       </c>
       <c r="E3" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>2026-10-21 08:30:00</v>
       </c>
       <c r="F3" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="4">
@@ -475,16 +475,16 @@
         <v>OLAM-9292-ST8F</v>
       </c>
       <c r="C4" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Quemada / Ya Usada</v>
       </c>
       <c r="D4" t="str">
-        <v>DISPONIBLE</v>
+        <v>Ana Lucia Marroquin</v>
       </c>
       <c r="E4" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>2026-10-21 08:45:00</v>
       </c>
       <c r="F4" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="5">
@@ -495,16 +495,16 @@
         <v>OLAM-TXTE-CB62</v>
       </c>
       <c r="C5" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Quemada / Ya Usada</v>
       </c>
       <c r="D5" t="str">
-        <v>DISPONIBLE</v>
+        <v>Jessica Noriega</v>
       </c>
       <c r="E5" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>2026-10-21 09:00:00</v>
       </c>
       <c r="F5" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="6">
@@ -515,16 +515,16 @@
         <v>OLAM-XR4P-6C73</v>
       </c>
       <c r="C6" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Quemada / Ya Usada</v>
       </c>
       <c r="D6" t="str">
-        <v>DISPONIBLE</v>
+        <v>Wally Natareno</v>
       </c>
       <c r="E6" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>2026-10-21 09:15:00</v>
       </c>
       <c r="F6" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="7">
@@ -535,16 +535,16 @@
         <v>OLAM-BQ86-GMC2</v>
       </c>
       <c r="C7" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Quemada / Ya Usada</v>
       </c>
       <c r="D7" t="str">
-        <v>DISPONIBLE</v>
+        <v>Erick Curley</v>
       </c>
       <c r="E7" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>2026-10-21 09:30:00</v>
       </c>
       <c r="F7" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="8">
@@ -555,16 +555,16 @@
         <v>OLAM-ZDHF-TNK6</v>
       </c>
       <c r="C8" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Quemada / Ya Usada</v>
       </c>
       <c r="D8" t="str">
-        <v>DISPONIBLE</v>
+        <v>Estuardo Cordova</v>
       </c>
       <c r="E8" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>2026-10-21 09:45:00</v>
       </c>
       <c r="F8" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="9">
@@ -575,16 +575,16 @@
         <v>OLAM-T5Q3-3SPY</v>
       </c>
       <c r="C9" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Quemada / Ya Usada</v>
       </c>
       <c r="D9" t="str">
-        <v>DISPONIBLE</v>
+        <v>Karina Pineda</v>
       </c>
       <c r="E9" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>2026-10-21 10:00:00</v>
       </c>
       <c r="F9" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="10">
@@ -595,16 +595,16 @@
         <v>OLAM-6VN3-7GFZ</v>
       </c>
       <c r="C10" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Quemada / Ya Usada</v>
       </c>
       <c r="D10" t="str">
-        <v>DISPONIBLE</v>
+        <v>Klissman Hernandez</v>
       </c>
       <c r="E10" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>2026-10-21 10:15:00</v>
       </c>
       <c r="F10" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="11">
@@ -615,16 +615,16 @@
         <v>OLAM-4BAQ-FK83</v>
       </c>
       <c r="C11" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Quemada / Ya Usada</v>
       </c>
       <c r="D11" t="str">
-        <v>DISPONIBLE</v>
+        <v>Elio Caceros</v>
       </c>
       <c r="E11" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>2026-10-21 10:30:00</v>
       </c>
       <c r="F11" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="12">
@@ -635,16 +635,16 @@
         <v>OLAM-65JB-ZFA6</v>
       </c>
       <c r="C12" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Quemada / Ya Usada</v>
       </c>
       <c r="D12" t="str">
-        <v>DISPONIBLE</v>
+        <v>Josue Aguilar</v>
       </c>
       <c r="E12" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>2026-10-21 10:45:00</v>
       </c>
       <c r="F12" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="13">
@@ -655,16 +655,16 @@
         <v>OLAM-64Q9-9R3T</v>
       </c>
       <c r="C13" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Quemada / Ya Usada</v>
       </c>
       <c r="D13" t="str">
-        <v>DISPONIBLE</v>
+        <v>Elias Quiej</v>
       </c>
       <c r="E13" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>2026-10-21 11:00:00</v>
       </c>
       <c r="F13" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="14">
@@ -675,16 +675,16 @@
         <v>OLAM-SDB8-E3SP</v>
       </c>
       <c r="C14" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Disponible</v>
       </c>
       <c r="D14" t="str">
-        <v>DISPONIBLE</v>
+        <v>—</v>
       </c>
       <c r="E14" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>—</v>
       </c>
       <c r="F14" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="15">
@@ -695,16 +695,16 @@
         <v>OLAM-W57M-A7TV</v>
       </c>
       <c r="C15" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Disponible</v>
       </c>
       <c r="D15" t="str">
-        <v>DISPONIBLE</v>
+        <v>—</v>
       </c>
       <c r="E15" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>—</v>
       </c>
       <c r="F15" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="16">
@@ -715,16 +715,16 @@
         <v>OLAM-TDJR-RD6C</v>
       </c>
       <c r="C16" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Disponible</v>
       </c>
       <c r="D16" t="str">
-        <v>DISPONIBLE</v>
+        <v>—</v>
       </c>
       <c r="E16" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>—</v>
       </c>
       <c r="F16" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="17">
@@ -735,16 +735,16 @@
         <v>OLAM-Q4YQ-EKM4</v>
       </c>
       <c r="C17" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Disponible</v>
       </c>
       <c r="D17" t="str">
-        <v>DISPONIBLE</v>
+        <v>—</v>
       </c>
       <c r="E17" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>—</v>
       </c>
       <c r="F17" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="18">
@@ -755,16 +755,16 @@
         <v>OLAM-2G3H-BWHN</v>
       </c>
       <c r="C18" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Disponible</v>
       </c>
       <c r="D18" t="str">
-        <v>DISPONIBLE</v>
+        <v>—</v>
       </c>
       <c r="E18" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>—</v>
       </c>
       <c r="F18" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="19">
@@ -775,16 +775,16 @@
         <v>OLAM-YQTZ-MHWY</v>
       </c>
       <c r="C19" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Disponible</v>
       </c>
       <c r="D19" t="str">
-        <v>DISPONIBLE</v>
+        <v>—</v>
       </c>
       <c r="E19" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>—</v>
       </c>
       <c r="F19" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="20">
@@ -795,16 +795,16 @@
         <v>OLAM-R7A7-VYWB</v>
       </c>
       <c r="C20" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Disponible</v>
       </c>
       <c r="D20" t="str">
-        <v>DISPONIBLE</v>
+        <v>—</v>
       </c>
       <c r="E20" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>—</v>
       </c>
       <c r="F20" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="21">
@@ -815,16 +815,16 @@
         <v>OLAM-B44W-2AVU</v>
       </c>
       <c r="C21" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Disponible</v>
       </c>
       <c r="D21" t="str">
-        <v>DISPONIBLE</v>
+        <v>—</v>
       </c>
       <c r="E21" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>—</v>
       </c>
       <c r="F21" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="22">
@@ -835,16 +835,16 @@
         <v>OLAM-5DGY-JGC4</v>
       </c>
       <c r="C22" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Disponible</v>
       </c>
       <c r="D22" t="str">
-        <v>DISPONIBLE</v>
+        <v>—</v>
       </c>
       <c r="E22" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>—</v>
       </c>
       <c r="F22" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="23">
@@ -855,16 +855,16 @@
         <v>OLAM-TUDE-J2BC</v>
       </c>
       <c r="C23" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Disponible</v>
       </c>
       <c r="D23" t="str">
-        <v>DISPONIBLE</v>
+        <v>—</v>
       </c>
       <c r="E23" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>—</v>
       </c>
       <c r="F23" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="24">
@@ -875,16 +875,16 @@
         <v>OLAM-SH59-9EAS</v>
       </c>
       <c r="C24" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Disponible</v>
       </c>
       <c r="D24" t="str">
-        <v>DISPONIBLE</v>
+        <v>—</v>
       </c>
       <c r="E24" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>—</v>
       </c>
       <c r="F24" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="25">
@@ -895,16 +895,16 @@
         <v>OLAM-QFZ8-PUQB</v>
       </c>
       <c r="C25" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Disponible</v>
       </c>
       <c r="D25" t="str">
-        <v>DISPONIBLE</v>
+        <v>—</v>
       </c>
       <c r="E25" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>—</v>
       </c>
       <c r="F25" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="26">
@@ -915,16 +915,16 @@
         <v>OLAM-W4GW-QDHY</v>
       </c>
       <c r="C26" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Disponible</v>
       </c>
       <c r="D26" t="str">
-        <v>DISPONIBLE</v>
+        <v>—</v>
       </c>
       <c r="E26" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>—</v>
       </c>
       <c r="F26" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="27">
@@ -935,16 +935,16 @@
         <v>OLAM-ZZG4-MJCX</v>
       </c>
       <c r="C27" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Disponible</v>
       </c>
       <c r="D27" t="str">
-        <v>DISPONIBLE</v>
+        <v>—</v>
       </c>
       <c r="E27" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>—</v>
       </c>
       <c r="F27" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="28">
@@ -955,16 +955,16 @@
         <v>OLAM-Q54Q-3F3S</v>
       </c>
       <c r="C28" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Disponible</v>
       </c>
       <c r="D28" t="str">
-        <v>DISPONIBLE</v>
+        <v>—</v>
       </c>
       <c r="E28" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>—</v>
       </c>
       <c r="F28" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="29">
@@ -975,16 +975,16 @@
         <v>OLAM-PD8C-D2FR</v>
       </c>
       <c r="C29" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Disponible</v>
       </c>
       <c r="D29" t="str">
-        <v>DISPONIBLE</v>
+        <v>—</v>
       </c>
       <c r="E29" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>—</v>
       </c>
       <c r="F29" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="30">
@@ -995,16 +995,16 @@
         <v>OLAM-BFFJ-E3QT</v>
       </c>
       <c r="C30" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Disponible</v>
       </c>
       <c r="D30" t="str">
-        <v>DISPONIBLE</v>
+        <v>—</v>
       </c>
       <c r="E30" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>—</v>
       </c>
       <c r="F30" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="31">
@@ -1015,16 +1015,16 @@
         <v>OLAM-NC5J-NTUD</v>
       </c>
       <c r="C31" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Disponible</v>
       </c>
       <c r="D31" t="str">
-        <v>DISPONIBLE</v>
+        <v>—</v>
       </c>
       <c r="E31" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>—</v>
       </c>
       <c r="F31" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="32">
@@ -1035,16 +1035,16 @@
         <v>OLAM-RQ2F-E2ZE</v>
       </c>
       <c r="C32" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Disponible</v>
       </c>
       <c r="D32" t="str">
-        <v>DISPONIBLE</v>
+        <v>—</v>
       </c>
       <c r="E32" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>—</v>
       </c>
       <c r="F32" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="33">
@@ -1055,16 +1055,16 @@
         <v>OLAM-QCC7-GCJ2</v>
       </c>
       <c r="C33" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Disponible</v>
       </c>
       <c r="D33" t="str">
-        <v>DISPONIBLE</v>
+        <v>—</v>
       </c>
       <c r="E33" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>—</v>
       </c>
       <c r="F33" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="34">
@@ -1075,16 +1075,16 @@
         <v>OLAM-N3WW-QP7T</v>
       </c>
       <c r="C34" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Disponible</v>
       </c>
       <c r="D34" t="str">
-        <v>DISPONIBLE</v>
+        <v>—</v>
       </c>
       <c r="E34" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>—</v>
       </c>
       <c r="F34" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="35">
@@ -1095,16 +1095,16 @@
         <v>OLAM-F7X4-U7ZC</v>
       </c>
       <c r="C35" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Disponible</v>
       </c>
       <c r="D35" t="str">
-        <v>DISPONIBLE</v>
+        <v>—</v>
       </c>
       <c r="E35" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>—</v>
       </c>
       <c r="F35" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="36">
@@ -1115,16 +1115,16 @@
         <v>OLAM-PMEQ-ADZC</v>
       </c>
       <c r="C36" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Disponible</v>
       </c>
       <c r="D36" t="str">
-        <v>DISPONIBLE</v>
+        <v>—</v>
       </c>
       <c r="E36" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>—</v>
       </c>
       <c r="F36" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="37">
@@ -1135,16 +1135,16 @@
         <v>OLAM-86ZS-B9KY</v>
       </c>
       <c r="C37" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Disponible</v>
       </c>
       <c r="D37" t="str">
-        <v>DISPONIBLE</v>
+        <v>—</v>
       </c>
       <c r="E37" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>—</v>
       </c>
       <c r="F37" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="38">
@@ -1155,16 +1155,16 @@
         <v>OLAM-T2DU-CRNE</v>
       </c>
       <c r="C38" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Disponible</v>
       </c>
       <c r="D38" t="str">
-        <v>DISPONIBLE</v>
+        <v>—</v>
       </c>
       <c r="E38" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>—</v>
       </c>
       <c r="F38" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="39">
@@ -1175,16 +1175,16 @@
         <v>OLAM-RW9K-9JSU</v>
       </c>
       <c r="C39" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Disponible</v>
       </c>
       <c r="D39" t="str">
-        <v>DISPONIBLE</v>
+        <v>—</v>
       </c>
       <c r="E39" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>—</v>
       </c>
       <c r="F39" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="40">
@@ -1195,16 +1195,16 @@
         <v>OLAM-HJBG-B5Z8</v>
       </c>
       <c r="C40" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Disponible</v>
       </c>
       <c r="D40" t="str">
-        <v>DISPONIBLE</v>
+        <v>—</v>
       </c>
       <c r="E40" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>—</v>
       </c>
       <c r="F40" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="41">
@@ -1215,16 +1215,16 @@
         <v>OLAM-V92D-4ZW4</v>
       </c>
       <c r="C41" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Disponible</v>
       </c>
       <c r="D41" t="str">
-        <v>DISPONIBLE</v>
+        <v>—</v>
       </c>
       <c r="E41" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>—</v>
       </c>
       <c r="F41" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="42">
@@ -1235,16 +1235,16 @@
         <v>OLAM-AKW3-B52K</v>
       </c>
       <c r="C42" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Disponible</v>
       </c>
       <c r="D42" t="str">
-        <v>DISPONIBLE</v>
+        <v>—</v>
       </c>
       <c r="E42" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>—</v>
       </c>
       <c r="F42" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="43">
@@ -1255,16 +1255,16 @@
         <v>OLAM-3HEK-W8SB</v>
       </c>
       <c r="C43" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Disponible</v>
       </c>
       <c r="D43" t="str">
-        <v>DISPONIBLE</v>
+        <v>—</v>
       </c>
       <c r="E43" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>—</v>
       </c>
       <c r="F43" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="44">
@@ -1275,16 +1275,16 @@
         <v>OLAM-BTAS-F65G</v>
       </c>
       <c r="C44" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Disponible</v>
       </c>
       <c r="D44" t="str">
-        <v>DISPONIBLE</v>
+        <v>—</v>
       </c>
       <c r="E44" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>—</v>
       </c>
       <c r="F44" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="45">
@@ -1295,16 +1295,16 @@
         <v>OLAM-PTPK-X6K2</v>
       </c>
       <c r="C45" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Disponible</v>
       </c>
       <c r="D45" t="str">
-        <v>DISPONIBLE</v>
+        <v>—</v>
       </c>
       <c r="E45" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>—</v>
       </c>
       <c r="F45" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="46">
@@ -1315,16 +1315,16 @@
         <v>OLAM-2D4F-269R</v>
       </c>
       <c r="C46" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Disponible</v>
       </c>
       <c r="D46" t="str">
-        <v>DISPONIBLE</v>
+        <v>—</v>
       </c>
       <c r="E46" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>—</v>
       </c>
       <c r="F46" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="47">
@@ -1335,16 +1335,16 @@
         <v>OLAM-UD4M-85DY</v>
       </c>
       <c r="C47" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Disponible</v>
       </c>
       <c r="D47" t="str">
-        <v>DISPONIBLE</v>
+        <v>—</v>
       </c>
       <c r="E47" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>—</v>
       </c>
       <c r="F47" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="48">
@@ -1355,16 +1355,16 @@
         <v>OLAM-N2A6-38QS</v>
       </c>
       <c r="C48" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Disponible</v>
       </c>
       <c r="D48" t="str">
-        <v>DISPONIBLE</v>
+        <v>—</v>
       </c>
       <c r="E48" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>—</v>
       </c>
       <c r="F48" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="49">
@@ -1375,16 +1375,16 @@
         <v>OLAM-XC83-TN8G</v>
       </c>
       <c r="C49" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Disponible</v>
       </c>
       <c r="D49" t="str">
-        <v>DISPONIBLE</v>
+        <v>—</v>
       </c>
       <c r="E49" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>—</v>
       </c>
       <c r="F49" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="50">
@@ -1395,16 +1395,16 @@
         <v>OLAM-Z5UH-JEMX</v>
       </c>
       <c r="C50" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Disponible</v>
       </c>
       <c r="D50" t="str">
-        <v>DISPONIBLE</v>
+        <v>—</v>
       </c>
       <c r="E50" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>—</v>
       </c>
       <c r="F50" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
     <row r="51">
@@ -1415,16 +1415,16 @@
         <v>OLAM-2U2C-WX8U</v>
       </c>
       <c r="C51" t="str">
-        <v>Acceso Desechable (1 Solo Uso)</v>
+        <v>Disponible</v>
       </c>
       <c r="D51" t="str">
-        <v>DISPONIBLE</v>
+        <v>—</v>
       </c>
       <c r="E51" t="str">
-        <v>Vendedor o Administrador</v>
+        <v>—</v>
       </c>
       <c r="F51" t="str">
-        <v>Válida exactamente para 1 inicio de sesión. Al entrar al sistema queda invalidada automáticamente de forma permanente.</v>
+        <v>Acceso Único Vendedores Droguería El Olam</v>
       </c>
     </row>
   </sheetData>

</xml_diff>